<commit_message>
Suivi Excel : vues du jour vidéo par vidéo (onglet + graphique empilé)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018GHR7DgBCo6t9CmjY4kYNE
</commit_message>
<xml_diff>
--- a/suivi/Decode_suivi_actu.xlsx
+++ b/suivi/Decode_suivi_actu.xlsx
@@ -10,8 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jour par jour" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vidéos" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Évolution par vidéo" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stories" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="À lire" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vues du jour par vidéo" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stories" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="À lire" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -281,6 +282,108 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Vues des stories</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Stories'!B1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="FF8A1F"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Stories'!$A$2:$A$8</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Stories'!$B$2:$B$8</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
@@ -1297,7 +1400,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Vues des stories</a:t>
+              <a:t>Vues gagnées chaque jour, vidéo par vidéo</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -1306,35 +1409,129 @@
     <plotArea>
       <barChart>
         <barDir val="col"/>
-        <grouping val="clustered"/>
+        <grouping val="stacked"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Stories'!B1</f>
+              <f>'Vues du jour par vidéo'!B1</f>
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="FF8A1F"/>
-            </a:solidFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <cat>
             <numRef>
-              <f>'Stories'!$A$2:$A$8</f>
+              <f>'Vues du jour par vidéo'!$A$2</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Stories'!$B$2:$B$8</f>
+              <f>'Vues du jour par vidéo'!$B$2</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Vues du jour par vidéo'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Vues du jour par vidéo'!$A$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Vues du jour par vidéo'!$C$2</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Vues du jour par vidéo'!D1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Vues du jour par vidéo'!$A$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Vues du jour par vidéo'!$D$2</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'Vues du jour par vidéo'!E1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Vues du jour par vidéo'!$A$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Vues du jour par vidéo'!$E$2</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'Vues du jour par vidéo'!F1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Vues du jour par vidéo'!$A$2</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Vues du jour par vidéo'!$F$2</f>
             </numRef>
           </val>
         </ser>
         <gapWidth val="150"/>
+        <overlap val="100"/>
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
@@ -1358,21 +1555,6 @@
         <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t/>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -1579,6 +1761,33 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -2441,6 +2650,98 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Jour</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>⚠️ Contenu effrayant… ou pas</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>FLASH SPÉCIAL 🚨 550 000 ou 8</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">POV : ta mamie t'écrit « ma </t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>👻 On ne parle que des casseu</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">👑 Vendredi soir : Macron au </t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Total du jour</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B2" s="3">
+        <f>IF('Évolution par vidéo'!B2="","",'Évolution par vidéo'!B2)</f>
+        <v/>
+      </c>
+      <c r="C2" s="3">
+        <f>IF('Évolution par vidéo'!C2="","",'Évolution par vidéo'!C2)</f>
+        <v/>
+      </c>
+      <c r="D2" s="3">
+        <f>IF('Évolution par vidéo'!D2="","",'Évolution par vidéo'!D2)</f>
+        <v/>
+      </c>
+      <c r="E2" s="3">
+        <f>IF('Évolution par vidéo'!E2="","",'Évolution par vidéo'!E2)</f>
+        <v/>
+      </c>
+      <c r="F2" s="3">
+        <f>IF('Évolution par vidéo'!F2="","",'Évolution par vidéo'!F2)</f>
+        <v/>
+      </c>
+      <c r="G2" s="3">
+        <f>SUM(B2:F2)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2748,13 +3049,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2791,12 +3092,19 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>Taux d'engagement = (likes + commentaires + partages + enregistrements) / comptes touchés.</t>
+          <t>« Vues du jour par vidéo » = vues gagnées par chaque vidéo depuis le relevé de la veille.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Taux d'engagement = (likes + commentaires + partages + enregistrements) / comptes touchés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Les statistiques d'une story ne sont lisibles que pendant ses 24 h : dernier relevé conservé.</t>
         </is>

</xml_diff>